<commit_message>
Importación de productos: Agregar campo de Unidad de medida
</commit_message>
<xml_diff>
--- a/Backend/public/docs/productos-format.xlsx
+++ b/Backend/public/docs/productos-format.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jesus Alvarado\Documents\GitHub\Smartyme\Backend\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5062DA0E-D7AC-44D1-9ED1-68F29E4F334E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63EBB52D-6DEE-4E6E-A6B9-F2E711A7B2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,42 +33,45 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>Nombre</t>
-  </si>
-  <si>
-    <t>Precio</t>
-  </si>
-  <si>
-    <t>Costo</t>
-  </si>
-  <si>
-    <t>Categoria</t>
-  </si>
-  <si>
-    <t>Codigo</t>
-  </si>
-  <si>
-    <t>Descripcion</t>
-  </si>
-  <si>
-    <t>Marca</t>
-  </si>
-  <si>
-    <t>Codigo_de_barra</t>
-  </si>
-  <si>
-    <t>Proveedor_nombre</t>
-  </si>
-  <si>
-    <t>Proveedor_apellido</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>sucursal_1_stock</t>
   </si>
   <si>
     <t>sucursal_2_stock</t>
+  </si>
+  <si>
+    <t>nombre</t>
+  </si>
+  <si>
+    <t>precio</t>
+  </si>
+  <si>
+    <t>costo</t>
+  </si>
+  <si>
+    <t>categoria</t>
+  </si>
+  <si>
+    <t>codigo</t>
+  </si>
+  <si>
+    <t>descripcion</t>
+  </si>
+  <si>
+    <t>marca</t>
+  </si>
+  <si>
+    <t>unidad_medida</t>
+  </si>
+  <si>
+    <t>codigo_de_barra</t>
+  </si>
+  <si>
+    <t>proveedor_nombre</t>
+  </si>
+  <si>
+    <t>proveedor_apellido</t>
   </si>
 </sst>
 </file>
@@ -408,53 +411,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="4" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.109375" customWidth="1"/>
-    <col min="10" max="10" width="18.21875" customWidth="1"/>
-    <col min="11" max="11" width="18.6640625" customWidth="1"/>
-    <col min="12" max="12" width="17" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.109375" customWidth="1"/>
+    <col min="11" max="11" width="18.21875" customWidth="1"/>
+    <col min="12" max="12" width="18.6640625" customWidth="1"/>
+    <col min="13" max="13" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" t="s">
-        <v>9</v>
+      <c r="M1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SP-230: Solucionar como se refleja descuentos en los reportes de ventas
</commit_message>
<xml_diff>
--- a/Backend/public/docs/productos-format.xlsx
+++ b/Backend/public/docs/productos-format.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10209"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jesus Alvarado\Documents\GitHub\Smartyme\Backend\public\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dcamacho/David/smartpyme/Backend/public/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63EBB52D-6DEE-4E6E-A6B9-F2E711A7B2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099AAD3D-CAF0-0940-B72D-1BC894F8430F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="23260" windowHeight="13180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>sucursal_1_stock</t>
   </si>
@@ -72,17 +72,26 @@
   </si>
   <si>
     <t>proveedor_apellido</t>
+  </si>
+  <si>
+    <t>subcategoria</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -105,8 +114,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -411,18 +421,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="4" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.109375" customWidth="1"/>
-    <col min="11" max="11" width="18.21875" customWidth="1"/>
-    <col min="12" max="12" width="18.6640625" customWidth="1"/>
-    <col min="13" max="13" width="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.1640625" customWidth="1"/>
+    <col min="12" max="12" width="18.1640625" customWidth="1"/>
+    <col min="13" max="13" width="18.6640625" customWidth="1"/>
+    <col min="14" max="14" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -441,25 +451,28 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Planilla de productos, precio sin IVA
</commit_message>
<xml_diff>
--- a/Backend/public/docs/productos-format.xlsx
+++ b/Backend/public/docs/productos-format.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jesus Alvarado\Documents\GitHub\Smartyme\Backend\public\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ingal\Documentos\GitHub\smartpyme\Backend\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63EBB52D-6DEE-4E6E-A6B9-F2E711A7B2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99D88308-7F1D-4811-9F1B-5CC863E7A726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,9 +44,6 @@
     <t>nombre</t>
   </si>
   <si>
-    <t>precio</t>
-  </si>
-  <si>
     <t>costo</t>
   </si>
   <si>
@@ -72,6 +69,9 @@
   </si>
   <si>
     <t>proveedor_apellido</t>
+  </si>
+  <si>
+    <t>precio_sin_iva</t>
   </si>
 </sst>
 </file>
@@ -415,6 +415,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19.109375" customWidth="1"/>
     <col min="11" max="11" width="18.21875" customWidth="1"/>
@@ -427,10 +428,10 @@
         <v>2</v>
       </c>
       <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>4</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
@@ -439,28 +440,28 @@
         <v>1</v>
       </c>
       <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
descargar plantillas de servicios
</commit_message>
<xml_diff>
--- a/Backend/public/docs/productos-format.xlsx
+++ b/Backend/public/docs/productos-format.xlsx
@@ -1,49 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ingal\Documentos\GitHub\smartpyme\Backend\public\docs\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99D88308-7F1D-4811-9F1B-5CC863E7A726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
+    <sheet name="Importar productos" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029" forceFullCalc="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
-  <si>
-    <t>sucursal_1_stock</t>
-  </si>
-  <si>
-    <t>sucursal_2_stock</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
   <si>
     <t>nombre</t>
   </si>
   <si>
+    <t>precio_sin_iva</t>
+  </si>
+  <si>
     <t>costo</t>
   </si>
   <si>
@@ -59,6 +38,9 @@
     <t>marca</t>
   </si>
   <si>
+    <t>impuesto</t>
+  </si>
+  <si>
     <t>unidad_medida</t>
   </si>
   <si>
@@ -71,26 +53,52 @@
     <t>proveedor_apellido</t>
   </si>
   <si>
-    <t>precio_sin_iva</t>
+    <t>genera_comanda</t>
+  </si>
+  <si>
+    <t>destino_comanda</t>
+  </si>
+  <si>
+    <t>stock_1 - AS Analytics (AS Analytics)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -105,22 +113,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -410,61 +411,89 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:O1"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.109375" customWidth="1"/>
-    <col min="11" max="11" width="18.21875" customWidth="1"/>
-    <col min="12" max="12" width="18.6640625" customWidth="1"/>
-    <col min="13" max="13" width="17" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.141" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="6.998" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="11.711" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="8.141" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="6.998" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="10.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="9" max="9" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="11" max="11" width="19.995" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="22.28" bestFit="true" customWidth="true" style="0"/>
+    <col min="13" max="13" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="14" max="14" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="15" max="15" width="44.703" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:15">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" t="s">
-        <v>11</v>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>